<commit_message>
feat(creator-web): 店面改版為果醬罐 Neo-Brutalism 視覺
- base.css / list.css 換 v3 tokens（2px 墨線、軟投影、貼紙硬底影、Caveat 手寫）
- 依設計稿改版商店列表、作品頁、結帳成功/失敗、404；結帳頁與訂單下載頁延續同規範
- 共用元件對齊 portal-web：果醬罐 BrandLogo、墨黑滿版 footer、便條淡彩 ProductThumb、手繪貼紙 icon 系統
- 移除 RotatingWord / ResultArt 與深色主題；favicon 比照 portal-web
- 修正直接進入結帳頁 / Stripe 導回時購物車未載入目錄誤顯示為空
- i18n：result / notfound 文案依設計稿重寫，新增手寫註記等 key 並回寫 xlsx

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/creator-web/i18n.xlsx
+++ b/apps/creator-web/i18n.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="499">
   <si>
     <t>key</t>
   </si>
@@ -118,6 +118,9 @@
     <t>nav.searchTitle</t>
   </si>
   <si>
+    <t>nav.search</t>
+  </si>
+  <si>
     <t>nav.cartTitle</t>
   </si>
   <si>
@@ -289,6 +292,15 @@
     <t>Sheet music, photo collections, e-books — buy directly from the creator and download instantly after payment.</t>
   </si>
   <si>
+    <t>list.bannerAlt</t>
+  </si>
+  <si>
+    <t>{store} 的店面橫幅</t>
+  </si>
+  <si>
+    <t>{store} storefront banner</t>
+  </si>
+  <si>
     <t>list.statWorks</t>
   </si>
   <si>
@@ -511,54 +523,6 @@
     <t>New</t>
   </si>
   <si>
-    <t>follow.title</t>
-  </si>
-  <si>
-    <t>追蹤這位創作者</t>
-  </si>
-  <si>
-    <t>Follow this creator</t>
-  </si>
-  <si>
-    <t>follow.desc</t>
-  </si>
-  <si>
-    <t>新作品上架時通知你，免註冊。</t>
-  </si>
-  <si>
-    <t>Get notified when new work drops — no account needed.</t>
-  </si>
-  <si>
-    <t>follow.placeholder</t>
-  </si>
-  <si>
-    <t>輸入信箱</t>
-  </si>
-  <si>
-    <t>Your email</t>
-  </si>
-  <si>
-    <t>follow.cta</t>
-  </si>
-  <si>
-    <t>follow.submitting</t>
-  </si>
-  <si>
-    <t>follow.doneTitle</t>
-  </si>
-  <si>
-    <t>You're following</t>
-  </si>
-  <si>
-    <t>follow.doneDesc</t>
-  </si>
-  <si>
-    <t>新作品會寄到你的信箱。</t>
-  </si>
-  <si>
-    <t>New work will land in your inbox.</t>
-  </si>
-  <si>
     <t>spotlight.badge</t>
   </si>
   <si>
@@ -580,10 +544,16 @@
     <t>spotlight.cta</t>
   </si>
   <si>
-    <t>查看作品 →</t>
-  </si>
-  <si>
-    <t>View work →</t>
+    <t>查看作品</t>
+  </si>
+  <si>
+    <t>View work</t>
+  </si>
+  <si>
+    <t>spotlight.freeNote</t>
+  </si>
+  <si>
+    <t>free!</t>
   </si>
   <si>
     <t>detail.screenLabel</t>
@@ -643,10 +613,10 @@
     <t>detail.contentsTitle</t>
   </si>
   <si>
-    <t>內容物（{count} 個檔案）</t>
-  </si>
-  <si>
-    <t>Contents ({count} files)</t>
+    <t>內容物{count}</t>
+  </si>
+  <si>
+    <t>Contents{count}</t>
   </si>
   <si>
     <t>detail.getFree</t>
@@ -760,6 +730,30 @@
     <t>{count} 次</t>
   </si>
   <si>
+    <t>detail.contentsCount</t>
+  </si>
+  <si>
+    <t>（{count} 個檔案）</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ({count} files)</t>
+  </si>
+  <si>
+    <t>detail.favTitle</t>
+  </si>
+  <si>
+    <t>收藏</t>
+  </si>
+  <si>
+    <t>Save to favorites</t>
+  </si>
+  <si>
+    <t>detail.handNoteFree</t>
+  </si>
+  <si>
+    <t>grab it, it's free ♡</t>
+  </si>
+  <si>
     <t>review.title</t>
   </si>
   <si>
@@ -1120,34 +1114,319 @@
     <t>Checkout result</t>
   </si>
   <si>
-    <t>result.successOrder</t>
-  </si>
-  <si>
-    <t>訂單 {id}</t>
-  </si>
-  <si>
-    <t>Order {id}</t>
-  </si>
-  <si>
     <t>result.successTitle</t>
   </si>
   <si>
-    <t>購買完成</t>
-  </si>
-  <si>
-    <t>Purchase complete</t>
+    <t>付款成功，作品是你的了{punct}</t>
+  </si>
+  <si>
+    <t>Payment complete — it's yours{punct}</t>
+  </si>
+  <si>
+    <t>result.successPunct</t>
+  </si>
+  <si>
+    <t>！</t>
+  </si>
+  <si>
+    <t>!</t>
   </si>
   <si>
     <t>result.successSub</t>
   </si>
   <si>
-    <t>收據與下載連結已寄至 {email}</t>
-  </si>
-  <si>
-    <t>Your receipt and download link have been sent to {email}</t>
-  </si>
-  <si>
-    <t>result.download</t>
+    <t>下載連結同時寄到了 {email}，保留那封信隨時可以重新下載。</t>
+  </si>
+  <si>
+    <t>The download link was also sent to {email}. Keep that email to re-download any time.</t>
+  </si>
+  <si>
+    <t>result.orderNumber</t>
+  </si>
+  <si>
+    <t>訂單編號</t>
+  </si>
+  <si>
+    <t>Order no.</t>
+  </si>
+  <si>
+    <t>result.payMethod</t>
+  </si>
+  <si>
+    <t>以 Stripe 安全付款</t>
+  </si>
+  <si>
+    <t>Paid securely via Stripe</t>
+  </si>
+  <si>
+    <t>result.total</t>
+  </si>
+  <si>
+    <t>合計</t>
+  </si>
+  <si>
+    <t>result.downloadAll</t>
+  </si>
+  <si>
+    <t>下載作品</t>
+  </si>
+  <si>
+    <t>Download your work</t>
+  </si>
+  <si>
+    <t>result.backToStore</t>
+  </si>
+  <si>
+    <t>回到商店</t>
+  </si>
+  <si>
+    <t>Back to store</t>
+  </si>
+  <si>
+    <t>result.continueExplore</t>
+  </si>
+  <si>
+    <t>繼續逛市集</t>
+  </si>
+  <si>
+    <t>Keep exploring</t>
+  </si>
+  <si>
+    <t>result.handNoteSuccess</t>
+  </si>
+  <si>
+    <t>happy jamming ♪</t>
+  </si>
+  <si>
+    <t>result.successTitle2</t>
+  </si>
+  <si>
+    <t>付款完成</t>
+  </si>
+  <si>
+    <t>Payment complete</t>
+  </si>
+  <si>
+    <t>result.successSub2</t>
+  </si>
+  <si>
+    <t>收據與下載連結已寄至您的信箱。</t>
+  </si>
+  <si>
+    <t>Your receipt and download link have been sent to your email.</t>
+  </si>
+  <si>
+    <t>result.cancelTitle</t>
+  </si>
+  <si>
+    <t>付款沒有成功</t>
+  </si>
+  <si>
+    <t>Payment didn't go through</t>
+  </si>
+  <si>
+    <t>result.cancelSub</t>
+  </si>
+  <si>
+    <t>{keep}銀行的預授權（若有）會在幾天內自動釋放，你的購物車也原封不動。</t>
+  </si>
+  <si>
+    <t>{keep}Any bank pre-authorization will be released automatically within a few days, and your cart is untouched.</t>
+  </si>
+  <si>
+    <t>result.cancelKeep</t>
+  </si>
+  <si>
+    <t>放心，這筆交易沒有扣款。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Don't worry — you were not charged. </t>
+  </si>
+  <si>
+    <t>result.cartLabel</t>
+  </si>
+  <si>
+    <t>你的購物車</t>
+  </si>
+  <si>
+    <t>Your cart</t>
+  </si>
+  <si>
+    <t>result.cartKept</t>
+  </si>
+  <si>
+    <t>已保留</t>
+  </si>
+  <si>
+    <t>Saved</t>
+  </si>
+  <si>
+    <t>result.causesTitle</t>
+  </si>
+  <si>
+    <t>常見原因</t>
+  </si>
+  <si>
+    <t>Common causes</t>
+  </si>
+  <si>
+    <t>result.causes.0</t>
+  </si>
+  <si>
+    <t>卡片餘額不足，或超過單筆消費限額</t>
+  </si>
+  <si>
+    <t>Insufficient balance, or over the per-transaction limit</t>
+  </si>
+  <si>
+    <t>result.causes.1</t>
+  </si>
+  <si>
+    <t>銀行拒絕了這筆跨國 / 線上交易，可致電開卡銀行放行</t>
+  </si>
+  <si>
+    <t>Your bank declined this online / cross-border payment — a quick call can unblock it</t>
+  </si>
+  <si>
+    <t>result.causes.2</t>
+  </si>
+  <si>
+    <t>卡號、效期或安全碼輸入有誤</t>
+  </si>
+  <si>
+    <t>Card number, expiry date or CVC was mistyped</t>
+  </si>
+  <si>
+    <t>result.retryPay</t>
+  </si>
+  <si>
+    <t>重新嘗試付款</t>
+  </si>
+  <si>
+    <t>Try payment again</t>
+  </si>
+  <si>
+    <t>result.contactUs</t>
+  </si>
+  <si>
+    <t>聯絡我們</t>
+  </si>
+  <si>
+    <t>Contact us</t>
+  </si>
+  <si>
+    <t>result.handNoteCancel</t>
+  </si>
+  <si>
+    <t>no worries — your jam is waiting ♪</t>
+  </si>
+  <si>
+    <t>notfound.screenLabel</t>
+  </si>
+  <si>
+    <t>404 找不到頁面</t>
+  </si>
+  <si>
+    <t>404 Not found</t>
+  </si>
+  <si>
+    <t>notfound.title</t>
+  </si>
+  <si>
+    <t>這件作品不在架上</t>
+  </si>
+  <si>
+    <t>This work isn't on the shelf</t>
+  </si>
+  <si>
+    <t>notfound.sub</t>
+  </si>
+  <si>
+    <t>可能已被創作者下架、改了網址，或從來沒有存在過。到店裡逛逛其他作品吧——寶物通常藏在下一個轉角。</t>
+  </si>
+  <si>
+    <t>It may have been taken down, moved to a new URL, or never existed. Browse the rest of the store — treasures usually hide around the next corner.</t>
+  </si>
+  <si>
+    <t>notfound.backToStore</t>
+  </si>
+  <si>
+    <t>回到{store}</t>
+  </si>
+  <si>
+    <t>Back to {store}</t>
+  </si>
+  <si>
+    <t>notfound.backToMarket</t>
+  </si>
+  <si>
+    <t>逛整個市集</t>
+  </si>
+  <si>
+    <t>Browse the marketplace</t>
+  </si>
+  <si>
+    <t>notfound.help</t>
+  </si>
+  <si>
+    <t>需要協助？</t>
+  </si>
+  <si>
+    <t>Need help?</t>
+  </si>
+  <si>
+    <t>notfound.handNote</t>
+  </si>
+  <si>
+    <t>sold out? or never here… 🤔</t>
+  </si>
+  <si>
+    <t>storeError.noVersion</t>
+  </si>
+  <si>
+    <t>部分商品尚無可購買的版本，請稍後再試</t>
+  </si>
+  <si>
+    <t>Some items have no purchasable version yet, please try again later</t>
+  </si>
+  <si>
+    <t>storeError.noPaymentUrl</t>
+  </si>
+  <si>
+    <t>無法取得付款頁面網址</t>
+  </si>
+  <si>
+    <t>Couldn’t get the payment page URL</t>
+  </si>
+  <si>
+    <t>order.screenLabel</t>
+  </si>
+  <si>
+    <t>訂單下載頁</t>
+  </si>
+  <si>
+    <t>Order downloads</t>
+  </si>
+  <si>
+    <t>order.title</t>
+  </si>
+  <si>
+    <t>訂單下載</t>
+  </si>
+  <si>
+    <t>Your downloads</t>
+  </si>
+  <si>
+    <t>order.orderNumber</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>order.total</t>
+  </si>
+  <si>
+    <t>order.download</t>
   </si>
   <si>
     <t>下載</t>
@@ -1156,165 +1435,6 @@
     <t>Download</t>
   </si>
   <si>
-    <t>result.continueExplore</t>
-  </si>
-  <si>
-    <t>繼續探索</t>
-  </si>
-  <si>
-    <t>Keep exploring</t>
-  </si>
-  <si>
-    <t>result.downloadAll</t>
-  </si>
-  <si>
-    <t>下載全部</t>
-  </si>
-  <si>
-    <t>Download all</t>
-  </si>
-  <si>
-    <t>result.successTitle2</t>
-  </si>
-  <si>
-    <t>付款完成</t>
-  </si>
-  <si>
-    <t>Payment complete</t>
-  </si>
-  <si>
-    <t>result.successSub2</t>
-  </si>
-  <si>
-    <t>收據與下載連結已寄至您的信箱。</t>
-  </si>
-  <si>
-    <t>Your receipt and download link have been sent to your email.</t>
-  </si>
-  <si>
-    <t>result.cancelTitle</t>
-  </si>
-  <si>
-    <t>付款已取消</t>
-  </si>
-  <si>
-    <t>Payment cancelled</t>
-  </si>
-  <si>
-    <t>result.cancelSub</t>
-  </si>
-  <si>
-    <t>您的購物車仍保留著，隨時可以回來完成結帳。</t>
-  </si>
-  <si>
-    <t>Your cart is still saved — come back any time to finish checking out.</t>
-  </si>
-  <si>
-    <t>result.backToCheckout</t>
-  </si>
-  <si>
-    <t>回到結帳</t>
-  </si>
-  <si>
-    <t>Back to checkout</t>
-  </si>
-  <si>
-    <t>notfound.screenLabel</t>
-  </si>
-  <si>
-    <t>404 找不到頁面</t>
-  </si>
-  <si>
-    <t>404 Not found</t>
-  </si>
-  <si>
-    <t>notfound.title</t>
-  </si>
-  <si>
-    <t>這個頁面不在這個{market}裡</t>
-  </si>
-  <si>
-    <t>This page isn’t in this {market}</t>
-  </si>
-  <si>
-    <t>notfound.market</t>
-  </si>
-  <si>
-    <t>市集</t>
-  </si>
-  <si>
-    <t>marketplace</t>
-  </si>
-  <si>
-    <t>notfound.sub</t>
-  </si>
-  <si>
-    <t>你要找的作品或頁面可能已下架、搬家，或網址打錯了。</t>
-  </si>
-  <si>
-    <t>The work or page you’re looking for may have been removed, moved, or the URL is wrong.</t>
-  </si>
-  <si>
-    <t>notfound.backToMarket</t>
-  </si>
-  <si>
-    <t>回到 Open Jam 市集</t>
-  </si>
-  <si>
-    <t>Back to the Open Jam marketplace</t>
-  </si>
-  <si>
-    <t>storeError.noVersion</t>
-  </si>
-  <si>
-    <t>部分商品尚無可購買的版本，請稍後再試</t>
-  </si>
-  <si>
-    <t>Some items have no purchasable version yet, please try again later</t>
-  </si>
-  <si>
-    <t>storeError.noPaymentUrl</t>
-  </si>
-  <si>
-    <t>無法取得付款頁面網址</t>
-  </si>
-  <si>
-    <t>Couldn’t get the payment page URL</t>
-  </si>
-  <si>
-    <t>order.screenLabel</t>
-  </si>
-  <si>
-    <t>訂單下載頁</t>
-  </si>
-  <si>
-    <t>Order downloads</t>
-  </si>
-  <si>
-    <t>order.title</t>
-  </si>
-  <si>
-    <t>訂單下載</t>
-  </si>
-  <si>
-    <t>Your downloads</t>
-  </si>
-  <si>
-    <t>order.orderNumber</t>
-  </si>
-  <si>
-    <t>訂單編號</t>
-  </si>
-  <si>
-    <t>Order</t>
-  </si>
-  <si>
-    <t>order.total</t>
-  </si>
-  <si>
-    <t>order.download</t>
-  </si>
-  <si>
     <t>order.refresh</t>
   </si>
   <si>
@@ -1388,12 +1508,6 @@
   </si>
   <si>
     <t>order.backToStore</t>
-  </si>
-  <si>
-    <t>回到商店</t>
-  </si>
-  <si>
-    <t>Back to store</t>
   </si>
 </sst>
 </file>
@@ -1779,7 +1893,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C160"/>
+  <dimension ref="A1:C174"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -1934,527 +2048,527 @@
         <v>35</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="29" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="33" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="35" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="37" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="38" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="39" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="41" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="42" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="44" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="C44" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="45" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>128</v>
-      </c>
       <c r="C45" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="46" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="47" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="48" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="49" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="50" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="51" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="52" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="53" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="54" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="55" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C55" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="57" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="58" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="59" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="60" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="61" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C61" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="62" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2462,241 +2576,241 @@
         <v>176</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>51</v>
+        <v>177</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>52</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>54</v>
+        <v>180</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="65" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="66" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="67" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="68" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="69" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="70" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="71" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="72" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="73" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="74" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="75" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="76" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="77" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="78" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="79" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="80" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="81" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
     </row>
     <row r="82" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="83" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>238</v>
+        <v>222</v>
       </c>
     </row>
     <row r="84" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2718,15 +2832,15 @@
         <v>243</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
     </row>
     <row r="86" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>246</v>
@@ -2740,194 +2854,194 @@
         <v>248</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>232</v>
+        <v>249</v>
       </c>
     </row>
     <row r="88" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="89" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="90" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="91" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="92" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="93" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="94" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="95" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="96" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="97" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="98" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="99" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="100" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="101" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="102" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="103" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="104" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
     </row>
     <row r="105" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2935,318 +3049,318 @@
         <v>300</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="106" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B106" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="B106" s="2" t="s">
-        <v>301</v>
-      </c>
       <c r="C106" s="2" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
     </row>
     <row r="107" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="108" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="109" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="110" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="111" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="112" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="113" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="114" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="115" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="116" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="117" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="118" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="119" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="120" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="121" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="122" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="123" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="124" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="125" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="126" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="127" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="128" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="129" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="130" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="131" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="132" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="133" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>383</v>
+        <v>339</v>
       </c>
     </row>
     <row r="134" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3290,260 +3404,414 @@
         <v>394</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="138" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="B138" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="B138" s="2" t="s">
+      <c r="C138" s="2" t="s">
         <v>397</v>
-      </c>
-      <c r="C138" s="2" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="139" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="B139" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="B139" s="2" t="s">
+      <c r="C139" s="2" t="s">
         <v>400</v>
-      </c>
-      <c r="C139" s="2" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="140" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="B140" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="B140" s="2" t="s">
+      <c r="C140" s="2" t="s">
         <v>403</v>
-      </c>
-      <c r="C140" s="2" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="141" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="B141" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="B141" s="2" t="s">
+      <c r="C141" s="2" t="s">
         <v>406</v>
-      </c>
-      <c r="C141" s="2" t="s">
-        <v>407</v>
       </c>
     </row>
     <row r="142" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="B142" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="B142" s="2" t="s">
+      <c r="C142" s="2" t="s">
         <v>409</v>
-      </c>
-      <c r="C142" s="2" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="143" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B143" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="B143" s="2" t="s">
+      <c r="C143" s="2" t="s">
         <v>412</v>
-      </c>
-      <c r="C143" s="2" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="144" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="B144" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="B144" s="2" t="s">
+      <c r="C144" s="2" t="s">
         <v>415</v>
-      </c>
-      <c r="C144" s="2" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="145" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B145" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="B145" s="2" t="s">
+      <c r="C145" s="2" t="s">
         <v>418</v>
-      </c>
-      <c r="C145" s="2" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="146" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="B146" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="B146" s="2" t="s">
+      <c r="C146" s="2" t="s">
         <v>421</v>
-      </c>
-      <c r="C146" s="2" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="147" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="B147" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="B147" s="2" t="s">
+      <c r="C147" s="2" t="s">
         <v>424</v>
-      </c>
-      <c r="C147" s="2" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="148" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B148" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="B148" s="2" t="s">
+      <c r="C148" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="C148" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="149" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="B149" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="B149" s="2" t="s">
+      <c r="C149" s="2" t="s">
         <v>430</v>
-      </c>
-      <c r="C149" s="2" t="s">
-        <v>431</v>
       </c>
     </row>
     <row r="150" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="B150" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="B150" s="2" t="s">
-        <v>340</v>
-      </c>
       <c r="C150" s="2" t="s">
-        <v>341</v>
+        <v>433</v>
       </c>
     </row>
     <row r="151" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>379</v>
+        <v>435</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>380</v>
+        <v>435</v>
       </c>
     </row>
     <row r="152" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="153" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="154" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="155" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
     <row r="156" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="157" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="158" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="159" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="160" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="C166" s="2" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A167" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A168" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="B168" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A169" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A170" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="B170" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A171" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="B171" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A173" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C173" s="2" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A174" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>